<commit_message>
update spreadsheet with glady's requests, such as calrifier summary label sizing
</commit_message>
<xml_diff>
--- a/src/copy_n_launch_xlsx/data/xlsx/daily_blank.xlsx
+++ b/src/copy_n_launch_xlsx/data/xlsx/daily_blank.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\oolong\dev\copy-n-launch-xlsx\src\copy_n_launch_xlsx\data\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\software\copy_n_launch_xlsx-0.2.4-py312-windows11-x86_64\_internal\copy_n_launch_xlsx\data\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D22656-41B4-4B54-8A52-0596ADC5067C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6204D076-B3A0-48C3-9AE1-39F2965A9A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="755" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="755" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hourly" sheetId="3" r:id="rId1"/>
@@ -32,10 +32,10 @@
     <definedName name="aeration_basin_do_south_avg_handheld">'Basin DO'!$J$9</definedName>
     <definedName name="aeration_basin_do_south_avg_probes">'Basin DO'!$J$10</definedName>
     <definedName name="aeration_basin_tempature">Various!$R$18</definedName>
-    <definedName name="basin_flow_total">Clarifier!$C$30</definedName>
-    <definedName name="basin_total_flow">Clarifier!$C$30</definedName>
-    <definedName name="clarifier_flow_total">Clarifier!$C$32</definedName>
-    <definedName name="clarifier_underflow_total">Clarifier!$C$31</definedName>
+    <definedName name="basin_flow_total">Clarifier!$F$31</definedName>
+    <definedName name="basin_total_flow">Clarifier!$F$31</definedName>
+    <definedName name="clarifier_flow_total">Clarifier!$F$33</definedName>
+    <definedName name="clarifier_underflow_total">Clarifier!$F$32</definedName>
     <definedName name="date">Print!$C$2</definedName>
     <definedName name="inf_flow_avg">Hourly!$C$27</definedName>
     <definedName name="inf_flow_max">Hourly!$C$28</definedName>
@@ -1893,7 +1893,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="265">
+  <cellXfs count="269">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2457,6 +2457,66 @@
     <xf numFmtId="166" fontId="11" fillId="3" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="11" fillId="6" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="17" fillId="6" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="6" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="17" fillId="6" borderId="16" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="6" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="6" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="17" fillId="6" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="11" fillId="6" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="6" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="3" borderId="53" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="3" borderId="54" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="16" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="36" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="17" fillId="0" borderId="38" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="20" fontId="17" fillId="0" borderId="44" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="20" fontId="17" fillId="0" borderId="63" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="63" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2564,85 +2624,25 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="11" fillId="6" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="17" fillId="6" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="6" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="17" fillId="6" borderId="16" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="6" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="6" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="17" fillId="6" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="11" fillId="6" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="6" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="60" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="46" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="59" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="60" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="53" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="19" fillId="3" borderId="53" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="3" borderId="54" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="17" fillId="6" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="19" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="16" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="36" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="17" fillId="0" borderId="38" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="59" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="20" fontId="17" fillId="0" borderId="44" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="20" fontId="17" fillId="0" borderId="63" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="63" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="57" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="40" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="57" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="56" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Comma 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -2967,7 +2967,7 @@
   <dimension ref="B2:Y35"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.42578125" style="62" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" style="62" customWidth="1"/>
     <col min="2" max="2" width="10.85546875" style="62" customWidth="1"/>
     <col min="3" max="3" width="12.28515625" style="62" customWidth="1"/>
     <col min="4" max="4" width="11.28515625" style="62" customWidth="1"/>
@@ -3645,7 +3645,7 @@
       <c r="B27" s="144" t="s">
         <v>18</v>
       </c>
-      <c r="C27" s="239" t="str">
+      <c r="C27" s="204" t="str">
         <f>IFERROR(AVERAGE(C3:C26),"Empty")</f>
         <v>Empty</v>
       </c>
@@ -3665,7 +3665,7 @@
         <f t="shared" si="0"/>
         <v>Empty</v>
       </c>
-      <c r="H27" s="239" t="str">
+      <c r="H27" s="204" t="str">
         <f t="shared" si="0"/>
         <v>Empty</v>
       </c>
@@ -3723,7 +3723,7 @@
       <c r="B28" s="145" t="s">
         <v>20</v>
       </c>
-      <c r="C28" s="239">
+      <c r="C28" s="204">
         <f>MAX(C3:C26)</f>
         <v>0</v>
       </c>
@@ -3773,7 +3773,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Q28" s="239">
+      <c r="Q28" s="204">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -3887,7 +3887,7 @@
       <c r="N30" s="165"/>
       <c r="O30" s="165"/>
       <c r="P30" s="165"/>
-      <c r="Q30" s="241">
+      <c r="Q30" s="206">
         <f t="shared" ref="Q30" si="3">SUM(Q$3:Q$26)</f>
         <v>0</v>
       </c>
@@ -4931,7 +4931,7 @@
       </c>
       <c r="G38" s="4">
         <f ca="1">NOW()-ROUNDDOWN(NOW(),0)</f>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -4951,7 +4951,7 @@
       </c>
       <c r="G39" s="4">
         <f t="shared" ref="G39:G82" ca="1" si="1">NOW()-ROUNDDOWN(NOW(),0)</f>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
@@ -4971,7 +4971,7 @@
       </c>
       <c r="G40" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
@@ -4991,7 +4991,7 @@
       </c>
       <c r="G41" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
@@ -5012,7 +5012,7 @@
       </c>
       <c r="G42" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="G43" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
@@ -5054,7 +5054,7 @@
       </c>
       <c r="G44" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
@@ -5075,7 +5075,7 @@
       </c>
       <c r="G45" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
@@ -5096,7 +5096,7 @@
       </c>
       <c r="G46" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
@@ -5117,7 +5117,7 @@
       </c>
       <c r="G47" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
@@ -5138,7 +5138,7 @@
       </c>
       <c r="G48" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -5159,7 +5159,7 @@
       </c>
       <c r="G49" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
@@ -5179,7 +5179,7 @@
       </c>
       <c r="G50" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
@@ -5199,7 +5199,7 @@
       </c>
       <c r="G51" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
@@ -5219,7 +5219,7 @@
       </c>
       <c r="G52" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="G53" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
@@ -5261,7 +5261,7 @@
       </c>
       <c r="G54" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
@@ -5282,7 +5282,7 @@
       </c>
       <c r="G55" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
@@ -5303,7 +5303,7 @@
       </c>
       <c r="G56" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
@@ -5324,7 +5324,7 @@
       </c>
       <c r="G57" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
@@ -5345,7 +5345,7 @@
       </c>
       <c r="G58" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
@@ -5366,7 +5366,7 @@
       </c>
       <c r="G59" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
@@ -5387,7 +5387,7 @@
       </c>
       <c r="G60" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="G61" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
@@ -5427,7 +5427,7 @@
       </c>
       <c r="G62" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
@@ -5447,7 +5447,7 @@
       </c>
       <c r="G63" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
@@ -5468,7 +5468,7 @@
       </c>
       <c r="G64" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
@@ -5489,7 +5489,7 @@
       </c>
       <c r="G65" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="G66" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
@@ -5531,7 +5531,7 @@
       </c>
       <c r="G67" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
@@ -5552,7 +5552,7 @@
       </c>
       <c r="G68" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
@@ -5573,7 +5573,7 @@
       </c>
       <c r="G69" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="G70" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
@@ -5615,7 +5615,7 @@
       </c>
       <c r="G71" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
@@ -5636,7 +5636,7 @@
       </c>
       <c r="G72" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
@@ -5656,7 +5656,7 @@
       </c>
       <c r="G73" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
@@ -5676,7 +5676,7 @@
       </c>
       <c r="G74" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
@@ -5696,7 +5696,7 @@
       </c>
       <c r="G75" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
@@ -5717,7 +5717,7 @@
       </c>
       <c r="G76" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
@@ -5738,7 +5738,7 @@
       </c>
       <c r="G77" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
@@ -5759,7 +5759,7 @@
       </c>
       <c r="G78" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
@@ -5780,7 +5780,7 @@
       </c>
       <c r="G79" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
@@ -5801,7 +5801,7 @@
       </c>
       <c r="G80" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
@@ -5822,7 +5822,7 @@
       </c>
       <c r="G81" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
@@ -5843,7 +5843,7 @@
       </c>
       <c r="G82" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
@@ -5866,7 +5866,7 @@
       </c>
       <c r="G83" s="4">
         <f t="shared" ref="G83:G114" ca="1" si="2">NOW()-ROUNDDOWN(NOW(),0)</f>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H83" s="1" t="s">
         <v>171</v>
@@ -5892,7 +5892,7 @@
       </c>
       <c r="G84" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H84" s="1" t="s">
         <v>171</v>
@@ -5918,7 +5918,7 @@
       </c>
       <c r="G85" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H85" s="1" t="s">
         <v>171</v>
@@ -5944,7 +5944,7 @@
       </c>
       <c r="G86" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H86" s="1" t="s">
         <v>171</v>
@@ -5970,7 +5970,7 @@
       </c>
       <c r="G87" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H87" s="1" t="s">
         <v>171</v>
@@ -5996,7 +5996,7 @@
       </c>
       <c r="G88" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H88" s="1" t="s">
         <v>171</v>
@@ -6022,7 +6022,7 @@
       </c>
       <c r="G89" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H89" s="1" t="s">
         <v>171</v>
@@ -6048,7 +6048,7 @@
       </c>
       <c r="G90" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H90" s="1" t="s">
         <v>171</v>
@@ -6074,7 +6074,7 @@
       </c>
       <c r="G91" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H91" s="1" t="s">
         <v>171</v>
@@ -6100,7 +6100,7 @@
       </c>
       <c r="G92" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H92" s="1" t="s">
         <v>171</v>
@@ -6126,7 +6126,7 @@
       </c>
       <c r="G93" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H93" s="1" t="s">
         <v>171</v>
@@ -6152,7 +6152,7 @@
       </c>
       <c r="G94" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H94" s="1" t="s">
         <v>171</v>
@@ -6178,7 +6178,7 @@
       </c>
       <c r="G95" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H95" s="1" t="s">
         <v>171</v>
@@ -6204,7 +6204,7 @@
       </c>
       <c r="G96" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H96" s="1" t="s">
         <v>171</v>
@@ -6230,7 +6230,7 @@
       </c>
       <c r="G97" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H97" s="1" t="s">
         <v>185</v>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="G98" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H98" s="1" t="s">
         <v>185</v>
@@ -6282,7 +6282,7 @@
       </c>
       <c r="G99" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H99" s="1" t="s">
         <v>185</v>
@@ -6308,7 +6308,7 @@
       </c>
       <c r="G100" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H100" s="1" t="s">
         <v>185</v>
@@ -6334,7 +6334,7 @@
       </c>
       <c r="G101" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H101" s="1" t="s">
         <v>185</v>
@@ -6360,7 +6360,7 @@
       </c>
       <c r="G102" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H102" s="1" t="s">
         <v>185</v>
@@ -6386,7 +6386,7 @@
       </c>
       <c r="G103" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H103" s="1" t="s">
         <v>185</v>
@@ -6412,7 +6412,7 @@
       </c>
       <c r="G104" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H104" s="1" t="s">
         <v>185</v>
@@ -6438,7 +6438,7 @@
       </c>
       <c r="G105" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H105" s="1" t="s">
         <v>185</v>
@@ -6464,7 +6464,7 @@
       </c>
       <c r="G106" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H106" s="1" t="s">
         <v>185</v>
@@ -6490,7 +6490,7 @@
       </c>
       <c r="G107" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H107" s="1" t="s">
         <v>185</v>
@@ -6516,7 +6516,7 @@
       </c>
       <c r="G108" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H108" s="1" t="s">
         <v>185</v>
@@ -6542,7 +6542,7 @@
       </c>
       <c r="G109" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H109" s="1" t="s">
         <v>185</v>
@@ -6568,7 +6568,7 @@
       </c>
       <c r="G110" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H110" s="1" t="s">
         <v>185</v>
@@ -6591,7 +6591,7 @@
       </c>
       <c r="G111" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.25">
@@ -6611,7 +6611,7 @@
       </c>
       <c r="G112" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
@@ -6631,7 +6631,7 @@
       </c>
       <c r="G113" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
@@ -6651,7 +6651,7 @@
       </c>
       <c r="G114" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
@@ -6671,7 +6671,7 @@
       </c>
       <c r="G115" s="4">
         <f t="shared" ref="G115:G146" ca="1" si="3">NOW()-ROUNDDOWN(NOW(),0)</f>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
@@ -6694,7 +6694,7 @@
       </c>
       <c r="G116" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
@@ -6717,7 +6717,7 @@
       </c>
       <c r="G117" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
@@ -6740,7 +6740,7 @@
       </c>
       <c r="G118" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
@@ -6763,7 +6763,7 @@
       </c>
       <c r="G119" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
@@ -6786,7 +6786,7 @@
       </c>
       <c r="G120" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
@@ -6809,7 +6809,7 @@
       </c>
       <c r="G121" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
@@ -6832,7 +6832,7 @@
       </c>
       <c r="G122" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.25">
@@ -6855,7 +6855,7 @@
       </c>
       <c r="G123" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.25">
@@ -6878,7 +6878,7 @@
       </c>
       <c r="G124" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.25">
@@ -6901,7 +6901,7 @@
       </c>
       <c r="G125" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.25">
@@ -6924,7 +6924,7 @@
       </c>
       <c r="G126" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.25">
@@ -6947,7 +6947,7 @@
       </c>
       <c r="G127" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.25">
@@ -6970,7 +6970,7 @@
       </c>
       <c r="G128" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.25">
@@ -6996,7 +6996,7 @@
       </c>
       <c r="G129" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.25">
@@ -7022,7 +7022,7 @@
       </c>
       <c r="G130" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.25">
@@ -7048,7 +7048,7 @@
       </c>
       <c r="G131" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.25">
@@ -7074,7 +7074,7 @@
       </c>
       <c r="G132" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.25">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="G133" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.25">
@@ -7126,7 +7126,7 @@
       </c>
       <c r="G134" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.25">
@@ -7152,7 +7152,7 @@
       </c>
       <c r="G135" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.25">
@@ -7178,7 +7178,7 @@
       </c>
       <c r="G136" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.25">
@@ -7204,7 +7204,7 @@
       </c>
       <c r="G137" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.25">
@@ -7230,7 +7230,7 @@
       </c>
       <c r="G138" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.25">
@@ -7256,7 +7256,7 @@
       </c>
       <c r="G139" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.25">
@@ -7282,7 +7282,7 @@
       </c>
       <c r="G140" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.25">
@@ -7308,7 +7308,7 @@
       </c>
       <c r="G141" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.25">
@@ -7334,7 +7334,7 @@
       </c>
       <c r="G142" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.25">
@@ -7360,7 +7360,7 @@
       </c>
       <c r="G143" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.25">
@@ -7386,7 +7386,7 @@
       </c>
       <c r="G144" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.25">
@@ -7412,7 +7412,7 @@
       </c>
       <c r="G145" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.25">
@@ -7438,7 +7438,7 @@
       </c>
       <c r="G146" s="4">
         <f t="shared" ca="1" si="3"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.25">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="G147" s="4">
         <f t="shared" ref="G147:G178" ca="1" si="4">NOW()-ROUNDDOWN(NOW(),0)</f>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.25">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="G148" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.25">
@@ -7516,7 +7516,7 @@
       </c>
       <c r="G149" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.25">
@@ -7542,7 +7542,7 @@
       </c>
       <c r="G150" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.25">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="G151" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.25">
@@ -7594,7 +7594,7 @@
       </c>
       <c r="G152" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.25">
@@ -7620,7 +7620,7 @@
       </c>
       <c r="G153" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.25">
@@ -7646,7 +7646,7 @@
       </c>
       <c r="G154" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.25">
@@ -7672,7 +7672,7 @@
       </c>
       <c r="G155" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.25">
@@ -7698,7 +7698,7 @@
       </c>
       <c r="G156" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.25">
@@ -7724,7 +7724,7 @@
       </c>
       <c r="G157" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.25">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="G158" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.25">
@@ -7776,7 +7776,7 @@
       </c>
       <c r="G159" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.25">
@@ -7802,7 +7802,7 @@
       </c>
       <c r="G160" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="161" spans="1:8" x14ac:dyDescent="0.25">
@@ -7828,7 +7828,7 @@
       </c>
       <c r="G161" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="162" spans="1:8" x14ac:dyDescent="0.25">
@@ -7854,7 +7854,7 @@
       </c>
       <c r="G162" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="163" spans="1:8" x14ac:dyDescent="0.25">
@@ -7880,7 +7880,7 @@
       </c>
       <c r="G163" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="164" spans="1:8" x14ac:dyDescent="0.25">
@@ -7906,7 +7906,7 @@
       </c>
       <c r="G164" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.25">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="G165" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="166" spans="1:8" x14ac:dyDescent="0.25">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="G166" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="167" spans="1:8" x14ac:dyDescent="0.25">
@@ -7975,7 +7975,7 @@
       </c>
       <c r="G167" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="168" spans="1:8" x14ac:dyDescent="0.25">
@@ -7998,7 +7998,7 @@
       </c>
       <c r="G168" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="169" spans="1:8" x14ac:dyDescent="0.25">
@@ -8021,7 +8021,7 @@
       </c>
       <c r="G169" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="170" spans="1:8" x14ac:dyDescent="0.25">
@@ -8044,7 +8044,7 @@
       </c>
       <c r="G170" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="171" spans="1:8" x14ac:dyDescent="0.25">
@@ -8067,7 +8067,7 @@
       </c>
       <c r="G171" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="172" spans="1:8" x14ac:dyDescent="0.25">
@@ -8090,7 +8090,7 @@
       </c>
       <c r="G172" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
       <c r="H172" s="8"/>
     </row>
@@ -8114,7 +8114,7 @@
       </c>
       <c r="G173" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="174" spans="1:8" x14ac:dyDescent="0.25">
@@ -8137,7 +8137,7 @@
       </c>
       <c r="G174" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="175" spans="1:8" x14ac:dyDescent="0.25">
@@ -8157,7 +8157,7 @@
       </c>
       <c r="G175" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="176" spans="1:8" x14ac:dyDescent="0.25">
@@ -8180,7 +8180,7 @@
       </c>
       <c r="G176" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="177" spans="1:7" x14ac:dyDescent="0.25">
@@ -8203,7 +8203,7 @@
       </c>
       <c r="G177" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="178" spans="1:7" x14ac:dyDescent="0.25">
@@ -8226,7 +8226,7 @@
       </c>
       <c r="G178" s="4">
         <f t="shared" ca="1" si="4"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="179" spans="1:7" x14ac:dyDescent="0.25">
@@ -8249,7 +8249,7 @@
       </c>
       <c r="G179" s="4">
         <f t="shared" ref="G179:G192" ca="1" si="5">NOW()-ROUNDDOWN(NOW(),0)</f>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="180" spans="1:7" x14ac:dyDescent="0.25">
@@ -8272,7 +8272,7 @@
       </c>
       <c r="G180" s="4">
         <f t="shared" ca="1" si="5"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="181" spans="1:7" x14ac:dyDescent="0.25">
@@ -8295,7 +8295,7 @@
       </c>
       <c r="G181" s="4">
         <f t="shared" ca="1" si="5"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="182" spans="1:7" x14ac:dyDescent="0.25">
@@ -8318,7 +8318,7 @@
       </c>
       <c r="G182" s="4">
         <f t="shared" ca="1" si="5"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="183" spans="1:7" x14ac:dyDescent="0.25">
@@ -8341,7 +8341,7 @@
       </c>
       <c r="G183" s="4">
         <f t="shared" ca="1" si="5"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="184" spans="1:7" x14ac:dyDescent="0.25">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="G184" s="4">
         <f t="shared" ca="1" si="5"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="185" spans="1:7" x14ac:dyDescent="0.25">
@@ -8387,7 +8387,7 @@
       </c>
       <c r="G185" s="4">
         <f t="shared" ca="1" si="5"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="186" spans="1:7" x14ac:dyDescent="0.25">
@@ -8410,7 +8410,7 @@
       </c>
       <c r="G186" s="4">
         <f t="shared" ca="1" si="5"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="187" spans="1:7" x14ac:dyDescent="0.25">
@@ -8433,7 +8433,7 @@
       </c>
       <c r="G187" s="4">
         <f t="shared" ca="1" si="5"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="188" spans="1:7" x14ac:dyDescent="0.25">
@@ -8456,7 +8456,7 @@
       </c>
       <c r="G188" s="4">
         <f t="shared" ca="1" si="5"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="189" spans="1:7" x14ac:dyDescent="0.25">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="G189" s="4">
         <f t="shared" ca="1" si="5"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="190" spans="1:7" x14ac:dyDescent="0.25">
@@ -8502,7 +8502,7 @@
       </c>
       <c r="G190" s="4">
         <f t="shared" ca="1" si="5"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="191" spans="1:7" x14ac:dyDescent="0.25">
@@ -8525,7 +8525,7 @@
       </c>
       <c r="G191" s="4">
         <f t="shared" ca="1" si="5"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="192" spans="1:7" x14ac:dyDescent="0.25">
@@ -8548,7 +8548,7 @@
       </c>
       <c r="G192" s="4">
         <f t="shared" ca="1" si="5"/>
-        <v>0.59909398148010951</v>
+        <v>0.70812858796125511</v>
       </c>
     </row>
     <row r="193" spans="1:7" x14ac:dyDescent="0.25">
@@ -9182,7 +9182,7 @@
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="237"/>
+      <c r="B4" s="202"/>
       <c r="C4" s="117" t="s">
         <v>257</v>
       </c>
@@ -9200,11 +9200,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="B1:AO32"/>
+  <dimension ref="B1:AO33"/>
   <sheetFormatPr defaultColWidth="5.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.5703125" style="36"/>
-    <col min="2" max="2" width="34" style="36" customWidth="1"/>
+    <col min="1" max="1" width="3.5703125" style="36" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" style="36" customWidth="1"/>
     <col min="3" max="9" width="7.7109375" style="36" customWidth="1"/>
     <col min="10" max="10" width="2.28515625" style="36" customWidth="1"/>
     <col min="11" max="13" width="7.7109375" style="36" customWidth="1"/>
@@ -9226,95 +9226,95 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:39" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="202"/>
-      <c r="C1" s="202"/>
-      <c r="D1" s="202"/>
-      <c r="E1" s="202"/>
-      <c r="F1" s="202"/>
-      <c r="G1" s="202"/>
-      <c r="H1" s="202"/>
-      <c r="I1" s="202"/>
-      <c r="J1" s="202"/>
-      <c r="K1" s="202"/>
-      <c r="L1" s="202"/>
-      <c r="M1" s="202"/>
-      <c r="N1" s="202"/>
-      <c r="O1" s="202"/>
-      <c r="P1" s="202"/>
-      <c r="Q1" s="202"/>
-      <c r="R1" s="202"/>
-      <c r="S1" s="202"/>
-      <c r="T1" s="202"/>
-      <c r="U1" s="202"/>
-      <c r="V1" s="202"/>
-      <c r="W1" s="202"/>
-      <c r="X1" s="202"/>
-      <c r="Y1" s="202"/>
-      <c r="Z1" s="202"/>
-      <c r="AA1" s="202"/>
-      <c r="AB1" s="202"/>
-      <c r="AC1" s="202"/>
-      <c r="AD1" s="202"/>
-      <c r="AE1" s="202"/>
-      <c r="AF1" s="202"/>
-      <c r="AG1" s="202"/>
-      <c r="AH1" s="202"/>
-      <c r="AI1" s="202"/>
-      <c r="AJ1" s="202"/>
-      <c r="AK1" s="202"/>
+      <c r="B1" s="223"/>
+      <c r="C1" s="223"/>
+      <c r="D1" s="223"/>
+      <c r="E1" s="223"/>
+      <c r="F1" s="223"/>
+      <c r="G1" s="223"/>
+      <c r="H1" s="223"/>
+      <c r="I1" s="223"/>
+      <c r="J1" s="223"/>
+      <c r="K1" s="223"/>
+      <c r="L1" s="223"/>
+      <c r="M1" s="223"/>
+      <c r="N1" s="223"/>
+      <c r="O1" s="223"/>
+      <c r="P1" s="223"/>
+      <c r="Q1" s="223"/>
+      <c r="R1" s="223"/>
+      <c r="S1" s="223"/>
+      <c r="T1" s="223"/>
+      <c r="U1" s="223"/>
+      <c r="V1" s="223"/>
+      <c r="W1" s="223"/>
+      <c r="X1" s="223"/>
+      <c r="Y1" s="223"/>
+      <c r="Z1" s="223"/>
+      <c r="AA1" s="223"/>
+      <c r="AB1" s="223"/>
+      <c r="AC1" s="223"/>
+      <c r="AD1" s="223"/>
+      <c r="AE1" s="223"/>
+      <c r="AF1" s="223"/>
+      <c r="AG1" s="223"/>
+      <c r="AH1" s="223"/>
+      <c r="AI1" s="223"/>
+      <c r="AJ1" s="223"/>
+      <c r="AK1" s="223"/>
     </row>
     <row r="2" spans="2:39" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="258"/>
-      <c r="C2" s="203" t="s">
+      <c r="B2" s="217"/>
+      <c r="C2" s="224" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="204"/>
-      <c r="E2" s="204"/>
-      <c r="F2" s="204"/>
-      <c r="G2" s="204"/>
-      <c r="H2" s="204"/>
-      <c r="I2" s="205"/>
+      <c r="D2" s="225"/>
+      <c r="E2" s="225"/>
+      <c r="F2" s="225"/>
+      <c r="G2" s="225"/>
+      <c r="H2" s="225"/>
+      <c r="I2" s="226"/>
       <c r="J2" s="104"/>
-      <c r="K2" s="203" t="s">
+      <c r="K2" s="224" t="s">
         <v>24</v>
       </c>
-      <c r="L2" s="204"/>
-      <c r="M2" s="204"/>
-      <c r="N2" s="204"/>
-      <c r="O2" s="204"/>
-      <c r="P2" s="204"/>
-      <c r="Q2" s="205"/>
+      <c r="L2" s="225"/>
+      <c r="M2" s="225"/>
+      <c r="N2" s="225"/>
+      <c r="O2" s="225"/>
+      <c r="P2" s="225"/>
+      <c r="Q2" s="226"/>
       <c r="R2" s="104"/>
-      <c r="S2" s="203" t="s">
+      <c r="S2" s="224" t="s">
         <v>25</v>
       </c>
-      <c r="T2" s="204"/>
-      <c r="U2" s="204"/>
-      <c r="V2" s="205"/>
+      <c r="T2" s="225"/>
+      <c r="U2" s="225"/>
+      <c r="V2" s="226"/>
       <c r="W2" s="104"/>
-      <c r="X2" s="203" t="s">
+      <c r="X2" s="224" t="s">
         <v>26</v>
       </c>
-      <c r="Y2" s="204"/>
-      <c r="Z2" s="204"/>
-      <c r="AA2" s="205"/>
+      <c r="Y2" s="225"/>
+      <c r="Z2" s="225"/>
+      <c r="AA2" s="226"/>
       <c r="AB2" s="104"/>
-      <c r="AC2" s="203" t="s">
+      <c r="AC2" s="224" t="s">
         <v>27</v>
       </c>
-      <c r="AD2" s="204"/>
-      <c r="AE2" s="204"/>
-      <c r="AF2" s="205"/>
+      <c r="AD2" s="225"/>
+      <c r="AE2" s="225"/>
+      <c r="AF2" s="226"/>
       <c r="AG2" s="104"/>
-      <c r="AH2" s="203" t="s">
+      <c r="AH2" s="224" t="s">
         <v>28</v>
       </c>
-      <c r="AI2" s="204"/>
-      <c r="AJ2" s="204"/>
-      <c r="AK2" s="205"/>
+      <c r="AI2" s="225"/>
+      <c r="AJ2" s="225"/>
+      <c r="AK2" s="226"/>
     </row>
     <row r="3" spans="2:39" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="259" t="s">
+      <c r="B3" s="218" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="37">
@@ -9414,7 +9414,7 @@
       </c>
     </row>
     <row r="4" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="B4" s="260">
+      <c r="B4" s="219">
         <v>0</v>
       </c>
       <c r="C4" s="44"/>
@@ -9456,7 +9456,7 @@
       <c r="AM4" s="52"/>
     </row>
     <row r="5" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="B5" s="261">
+      <c r="B5" s="220">
         <v>4.1666666666666664E-2</v>
       </c>
       <c r="C5" s="44"/>
@@ -9498,7 +9498,7 @@
       <c r="AM5" s="52"/>
     </row>
     <row r="6" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="B6" s="261">
+      <c r="B6" s="220">
         <v>8.3333333333333301E-2</v>
       </c>
       <c r="C6" s="44"/>
@@ -9540,7 +9540,7 @@
       <c r="AM6" s="52"/>
     </row>
     <row r="7" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="B7" s="261">
+      <c r="B7" s="220">
         <v>0.125</v>
       </c>
       <c r="C7" s="44"/>
@@ -9582,7 +9582,7 @@
       <c r="AM7" s="52"/>
     </row>
     <row r="8" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="B8" s="261">
+      <c r="B8" s="220">
         <v>0.16666666666666699</v>
       </c>
       <c r="C8" s="44"/>
@@ -9624,7 +9624,7 @@
       <c r="AM8" s="52"/>
     </row>
     <row r="9" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="B9" s="261">
+      <c r="B9" s="220">
         <v>0.20833333333333301</v>
       </c>
       <c r="C9" s="44"/>
@@ -9666,7 +9666,7 @@
       <c r="AM9" s="52"/>
     </row>
     <row r="10" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="B10" s="261">
+      <c r="B10" s="220">
         <v>0.25</v>
       </c>
       <c r="C10" s="44"/>
@@ -9708,7 +9708,7 @@
       <c r="AM10" s="52"/>
     </row>
     <row r="11" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="B11" s="261">
+      <c r="B11" s="220">
         <v>0.29166666666666702</v>
       </c>
       <c r="C11" s="44"/>
@@ -9750,7 +9750,7 @@
       <c r="AM11" s="52"/>
     </row>
     <row r="12" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="B12" s="261">
+      <c r="B12" s="220">
         <v>0.33333333333333298</v>
       </c>
       <c r="C12" s="44"/>
@@ -9792,7 +9792,7 @@
       <c r="AM12" s="52"/>
     </row>
     <row r="13" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="B13" s="261">
+      <c r="B13" s="220">
         <v>0.375</v>
       </c>
       <c r="C13" s="44"/>
@@ -9834,7 +9834,7 @@
       <c r="AM13" s="52"/>
     </row>
     <row r="14" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="B14" s="261">
+      <c r="B14" s="220">
         <v>0.41666666666666702</v>
       </c>
       <c r="C14" s="44"/>
@@ -9876,7 +9876,7 @@
       <c r="AM14" s="52"/>
     </row>
     <row r="15" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="B15" s="261">
+      <c r="B15" s="220">
         <v>0.45833333333333331</v>
       </c>
       <c r="C15" s="44"/>
@@ -9918,7 +9918,7 @@
       <c r="AM15" s="52"/>
     </row>
     <row r="16" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="B16" s="261">
+      <c r="B16" s="220">
         <v>0.5</v>
       </c>
       <c r="C16" s="44"/>
@@ -9958,7 +9958,7 @@
       <c r="AK16" s="46"/>
     </row>
     <row r="17" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B17" s="261">
+      <c r="B17" s="220">
         <v>0.54166666666666696</v>
       </c>
       <c r="C17" s="44"/>
@@ -9998,7 +9998,7 @@
       <c r="AK17" s="46"/>
     </row>
     <row r="18" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B18" s="261">
+      <c r="B18" s="220">
         <v>0.58333333333333337</v>
       </c>
       <c r="C18" s="44"/>
@@ -10040,7 +10040,7 @@
       <c r="AM18" s="52"/>
     </row>
     <row r="19" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B19" s="261">
+      <c r="B19" s="220">
         <v>0.625</v>
       </c>
       <c r="C19" s="44"/>
@@ -10083,7 +10083,7 @@
       <c r="AN19" s="56"/>
     </row>
     <row r="20" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B20" s="261">
+      <c r="B20" s="220">
         <v>0.66666666666666696</v>
       </c>
       <c r="C20" s="44"/>
@@ -10123,7 +10123,7 @@
       <c r="AK20" s="55"/>
     </row>
     <row r="21" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B21" s="261">
+      <c r="B21" s="220">
         <v>0.70833333333333304</v>
       </c>
       <c r="C21" s="44"/>
@@ -10167,7 +10167,7 @@
       <c r="AO21" s="56"/>
     </row>
     <row r="22" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B22" s="261">
+      <c r="B22" s="220">
         <v>0.75</v>
       </c>
       <c r="C22" s="44"/>
@@ -10211,7 +10211,7 @@
       <c r="AO22" s="56"/>
     </row>
     <row r="23" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B23" s="261">
+      <c r="B23" s="220">
         <v>0.79166666666666696</v>
       </c>
       <c r="C23" s="44"/>
@@ -10255,7 +10255,7 @@
       <c r="AO23" s="56"/>
     </row>
     <row r="24" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B24" s="261">
+      <c r="B24" s="220">
         <v>0.83333333333333304</v>
       </c>
       <c r="C24" s="44"/>
@@ -10299,7 +10299,7 @@
       <c r="AO24" s="56"/>
     </row>
     <row r="25" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B25" s="261">
+      <c r="B25" s="220">
         <v>0.875</v>
       </c>
       <c r="C25" s="44"/>
@@ -10343,7 +10343,7 @@
       <c r="AO25" s="56"/>
     </row>
     <row r="26" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B26" s="261">
+      <c r="B26" s="220">
         <v>0.91666666666666696</v>
       </c>
       <c r="C26" s="44"/>
@@ -10387,7 +10387,7 @@
       <c r="AO26" s="56"/>
     </row>
     <row r="27" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B27" s="262">
+      <c r="B27" s="221">
         <v>0.95833333333333304</v>
       </c>
       <c r="C27" s="44"/>
@@ -10431,34 +10431,34 @@
       <c r="AO27" s="56"/>
     </row>
     <row r="28" spans="2:41" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="263" t="s">
+      <c r="B28" s="222" t="s">
         <v>18</v>
       </c>
-      <c r="C28" s="257" t="str">
+      <c r="C28" s="216" t="str">
         <f>IFERROR(AVERAGEA(C$4:C$27),"Empty")</f>
         <v>Empty</v>
       </c>
-      <c r="D28" s="254" t="str">
+      <c r="D28" s="214" t="str">
         <f>IFERROR(AVERAGEA(D$4:D$27),"Empty")</f>
         <v>Empty</v>
       </c>
-      <c r="E28" s="254" t="str">
+      <c r="E28" s="214" t="str">
         <f>IFERROR(AVERAGEA(E$4:E$27),"Empty")</f>
         <v>Empty</v>
       </c>
-      <c r="F28" s="254" t="str">
+      <c r="F28" s="214" t="str">
         <f>IFERROR(AVERAGEA(F$4:F$27),"Empty")</f>
         <v>Empty</v>
       </c>
-      <c r="G28" s="254" t="str">
+      <c r="G28" s="214" t="str">
         <f>IFERROR(AVERAGEA(G$4:G$27),"Empty")</f>
         <v>Empty</v>
       </c>
-      <c r="H28" s="254" t="str">
+      <c r="H28" s="214" t="str">
         <f t="shared" ref="H28:I28" si="0">IFERROR(AVERAGEA(H$4:H$27),"Empty")</f>
         <v>Empty</v>
       </c>
-      <c r="I28" s="255" t="str">
+      <c r="I28" s="215" t="str">
         <f t="shared" si="0"/>
         <v>Empty</v>
       </c>
@@ -10560,8 +10560,8 @@
         <v>Empty</v>
       </c>
     </row>
-    <row r="29" spans="2:41" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="264" t="s">
+    <row r="29" spans="2:41" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="222" t="s">
         <v>271</v>
       </c>
       <c r="C29" s="174">
@@ -10690,37 +10690,84 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B30" s="252" t="s">
+    <row r="30" spans="2:41" s="264" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="265"/>
+      <c r="C30" s="187"/>
+      <c r="D30" s="187"/>
+      <c r="E30" s="187"/>
+      <c r="F30" s="187"/>
+      <c r="G30" s="187"/>
+      <c r="H30" s="187"/>
+      <c r="I30" s="187"/>
+      <c r="J30" s="187"/>
+      <c r="K30" s="187"/>
+      <c r="L30" s="187"/>
+      <c r="M30" s="187"/>
+      <c r="N30" s="187"/>
+      <c r="O30" s="187"/>
+      <c r="P30" s="187"/>
+      <c r="Q30" s="187"/>
+      <c r="R30" s="187"/>
+      <c r="S30" s="187"/>
+      <c r="T30" s="187"/>
+      <c r="U30" s="187"/>
+      <c r="V30" s="187"/>
+      <c r="W30" s="187"/>
+      <c r="X30" s="187"/>
+      <c r="Y30" s="187"/>
+      <c r="Z30" s="187"/>
+      <c r="AA30" s="187"/>
+      <c r="AB30" s="187"/>
+      <c r="AC30" s="187"/>
+      <c r="AD30" s="187"/>
+      <c r="AE30" s="187"/>
+      <c r="AF30" s="187"/>
+      <c r="AG30" s="187"/>
+      <c r="AH30" s="187"/>
+      <c r="AI30" s="187"/>
+      <c r="AJ30" s="187"/>
+      <c r="AK30" s="187"/>
+    </row>
+    <row r="31" spans="2:41" x14ac:dyDescent="0.25">
+      <c r="B31" s="258"/>
+      <c r="C31" s="266"/>
+      <c r="D31" s="258"/>
+      <c r="E31" s="259" t="s">
         <v>29</v>
       </c>
-      <c r="C30" s="256">
+      <c r="F31" s="209">
         <f>IFERROR(SUM(C29:Q29),"Empty")</f>
         <v>0</v>
       </c>
-      <c r="AE30" s="59"/>
-    </row>
-    <row r="31" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B31" s="252" t="s">
+      <c r="AH31" s="59"/>
+    </row>
+    <row r="32" spans="2:41" x14ac:dyDescent="0.25">
+      <c r="B32" s="260"/>
+      <c r="C32" s="267"/>
+      <c r="D32" s="260"/>
+      <c r="E32" s="261" t="s">
         <v>269</v>
       </c>
-      <c r="C31" s="244">
+      <c r="F32" s="209">
         <f>IFERROR(SUM(AC28:AK28),"Empty")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B32" s="253" t="s">
+    <row r="33" spans="2:34" x14ac:dyDescent="0.25">
+      <c r="B33" s="262"/>
+      <c r="C33" s="268"/>
+      <c r="D33" s="262"/>
+      <c r="E33" s="263" t="s">
         <v>270</v>
       </c>
-      <c r="C32" s="244">
+      <c r="F33" s="209">
         <f>IFERROR(SUM(S28:AA28),"Empty")</f>
         <v>0</v>
       </c>
-      <c r="F32" s="36" t="s">
+      <c r="I33" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="AE32" s="60" t="s">
+      <c r="AH33" s="60" t="s">
         <v>32</v>
       </c>
     </row>
@@ -10757,50 +10804,50 @@
   <sheetData>
     <row r="1" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="210" t="s">
+      <c r="B2" s="231" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="210" t="s">
+      <c r="C2" s="231" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="206" t="s">
+      <c r="D2" s="227" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="207"/>
-      <c r="F2" s="206" t="s">
+      <c r="E2" s="228"/>
+      <c r="F2" s="227" t="s">
         <v>36</v>
       </c>
-      <c r="G2" s="207"/>
-      <c r="H2" s="206" t="s">
+      <c r="G2" s="228"/>
+      <c r="H2" s="227" t="s">
         <v>37</v>
       </c>
-      <c r="I2" s="207"/>
-      <c r="J2" s="206" t="s">
+      <c r="I2" s="228"/>
+      <c r="J2" s="227" t="s">
         <v>38</v>
       </c>
-      <c r="K2" s="207"/>
-      <c r="L2" s="206" t="s">
+      <c r="K2" s="228"/>
+      <c r="L2" s="227" t="s">
         <v>39</v>
       </c>
-      <c r="M2" s="207"/>
+      <c r="M2" s="228"/>
     </row>
     <row r="3" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="211"/>
-      <c r="C3" s="211"/>
-      <c r="D3" s="208"/>
-      <c r="E3" s="209"/>
-      <c r="F3" s="208"/>
-      <c r="G3" s="209"/>
-      <c r="H3" s="208"/>
-      <c r="I3" s="209"/>
-      <c r="J3" s="208"/>
-      <c r="K3" s="209"/>
-      <c r="L3" s="208"/>
-      <c r="M3" s="209"/>
+      <c r="B3" s="232"/>
+      <c r="C3" s="232"/>
+      <c r="D3" s="229"/>
+      <c r="E3" s="230"/>
+      <c r="F3" s="229"/>
+      <c r="G3" s="230"/>
+      <c r="H3" s="229"/>
+      <c r="I3" s="230"/>
+      <c r="J3" s="229"/>
+      <c r="K3" s="230"/>
+      <c r="L3" s="229"/>
+      <c r="M3" s="230"/>
     </row>
     <row r="4" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="212"/>
-      <c r="C4" s="212"/>
+      <c r="B4" s="233"/>
+      <c r="C4" s="233"/>
       <c r="D4" s="169" t="s">
         <v>40</v>
       </c>
@@ -10994,7 +11041,7 @@
       <c r="C8" t="s">
         <v>264</v>
       </c>
-      <c r="D8" s="237" t="str">
+      <c r="D8" s="202" t="str">
         <f>IFERROR(AVERAGE(H6,L6,D6),"Empty")</f>
         <v>Empty</v>
       </c>
@@ -11005,7 +11052,7 @@
       <c r="C9" t="s">
         <v>265</v>
       </c>
-      <c r="D9" s="237" t="str">
+      <c r="D9" s="202" t="str">
         <f>IFERROR(AVERAGEA(J5,N5,F5),"Empty")</f>
         <v>Empty</v>
       </c>
@@ -11149,7 +11196,7 @@
       <c r="C18" t="s">
         <v>266</v>
       </c>
-      <c r="D18" s="237" t="str">
+      <c r="D18" s="202" t="str">
         <f>IFERROR(AVERAGE(H16,L16,D16),"Empty")</f>
         <v>Empty</v>
       </c>
@@ -11200,13 +11247,13 @@
       <c r="E2" s="117" t="s">
         <v>59</v>
       </c>
-      <c r="G2" s="213" t="s">
+      <c r="G2" s="234" t="s">
         <v>61</v>
       </c>
-      <c r="H2" s="214"/>
-      <c r="I2" s="214"/>
-      <c r="J2" s="214"/>
-      <c r="K2" s="215"/>
+      <c r="H2" s="235"/>
+      <c r="I2" s="235"/>
+      <c r="J2" s="235"/>
+      <c r="K2" s="236"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="119" t="s">
@@ -11302,13 +11349,13 @@
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="G8" s="216" t="s">
+      <c r="G8" s="237" t="s">
         <v>71</v>
       </c>
-      <c r="H8" s="216"/>
-      <c r="I8" s="216"/>
-      <c r="J8" s="216"/>
-      <c r="K8" s="245" t="str">
+      <c r="H8" s="237"/>
+      <c r="I8" s="237"/>
+      <c r="J8" s="237"/>
+      <c r="K8" s="210" t="str">
         <f>IFERROR(AVERAGE(H7:K7),"Empty")</f>
         <v>Empty</v>
       </c>
@@ -11333,7 +11380,7 @@
   <dimension ref="A1:AL37"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4" style="14" customWidth="1"/>
+    <col min="1" max="1" width="2.28515625" style="14" customWidth="1"/>
     <col min="2" max="2" width="11.42578125" style="14" customWidth="1"/>
     <col min="3" max="3" width="9.85546875" style="14" customWidth="1"/>
     <col min="4" max="4" width="5.42578125" style="14" customWidth="1"/>
@@ -11364,24 +11411,24 @@
   <sheetData>
     <row r="1" spans="2:38" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:38" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="220" t="s">
+      <c r="B2" s="241" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="221"/>
-      <c r="D2" s="221"/>
-      <c r="E2" s="221"/>
-      <c r="F2" s="221"/>
-      <c r="G2" s="221"/>
-      <c r="H2" s="222"/>
-      <c r="J2" s="223" t="s">
+      <c r="C2" s="242"/>
+      <c r="D2" s="242"/>
+      <c r="E2" s="242"/>
+      <c r="F2" s="242"/>
+      <c r="G2" s="242"/>
+      <c r="H2" s="243"/>
+      <c r="J2" s="244" t="s">
         <v>73</v>
       </c>
-      <c r="K2" s="224"/>
-      <c r="L2" s="225"/>
-      <c r="Q2" s="226" t="s">
+      <c r="K2" s="245"/>
+      <c r="L2" s="246"/>
+      <c r="Q2" s="247" t="s">
         <v>74</v>
       </c>
-      <c r="R2" s="227"/>
+      <c r="R2" s="248"/>
     </row>
     <row r="3" spans="2:38" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="17" t="s">
@@ -11548,20 +11595,20 @@
       <c r="W11" s="74"/>
     </row>
     <row r="12" spans="2:38" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="232" t="s">
+      <c r="B12" s="253" t="s">
         <v>90</v>
       </c>
-      <c r="C12" s="233"/>
-      <c r="D12" s="234"/>
-      <c r="E12" s="234"/>
-      <c r="F12" s="234"/>
-      <c r="G12" s="234"/>
-      <c r="H12" s="234"/>
-      <c r="I12" s="234"/>
-      <c r="J12" s="234"/>
-      <c r="K12" s="234"/>
-      <c r="L12" s="234"/>
-      <c r="M12" s="235"/>
+      <c r="C12" s="254"/>
+      <c r="D12" s="255"/>
+      <c r="E12" s="255"/>
+      <c r="F12" s="255"/>
+      <c r="G12" s="255"/>
+      <c r="H12" s="255"/>
+      <c r="I12" s="255"/>
+      <c r="J12" s="255"/>
+      <c r="K12" s="255"/>
+      <c r="L12" s="255"/>
+      <c r="M12" s="256"/>
       <c r="N12" s="74"/>
       <c r="P12" s="74"/>
       <c r="U12" s="100" t="s">
@@ -11580,20 +11627,20 @@
     <row r="13" spans="2:38" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="87"/>
       <c r="C13" s="88"/>
-      <c r="D13" s="228" t="s">
+      <c r="D13" s="249" t="s">
         <v>79</v>
       </c>
-      <c r="E13" s="228"/>
-      <c r="F13" s="228"/>
-      <c r="G13" s="228"/>
-      <c r="H13" s="228"/>
-      <c r="I13" s="229" t="s">
+      <c r="E13" s="249"/>
+      <c r="F13" s="249"/>
+      <c r="G13" s="249"/>
+      <c r="H13" s="249"/>
+      <c r="I13" s="250" t="s">
         <v>80</v>
       </c>
-      <c r="J13" s="230"/>
-      <c r="K13" s="230"/>
-      <c r="L13" s="230"/>
-      <c r="M13" s="231"/>
+      <c r="J13" s="251"/>
+      <c r="K13" s="251"/>
+      <c r="L13" s="251"/>
+      <c r="M13" s="252"/>
       <c r="P13" s="83"/>
       <c r="U13" s="101" t="s">
         <v>93</v>
@@ -11685,10 +11732,10 @@
         <v>Empty</v>
       </c>
       <c r="P16" s="30"/>
-      <c r="Q16" s="218" t="s">
+      <c r="Q16" s="239" t="s">
         <v>97</v>
       </c>
-      <c r="R16" s="219"/>
+      <c r="R16" s="240"/>
       <c r="U16" s="137" t="s">
         <v>98</v>
       </c>
@@ -11719,10 +11766,10 @@
         <v>Empty</v>
       </c>
       <c r="P17" s="30"/>
-      <c r="Q17" s="249" t="s">
+      <c r="Q17" s="213" t="s">
         <v>100</v>
       </c>
-      <c r="R17" s="247"/>
+      <c r="R17" s="211"/>
       <c r="U17" s="139" t="s">
         <v>101</v>
       </c>
@@ -11752,7 +11799,7 @@
       <c r="Q18" s="96" t="s">
         <v>261</v>
       </c>
-      <c r="R18" s="247"/>
+      <c r="R18" s="211"/>
       <c r="U18" s="25" t="s">
         <v>103</v>
       </c>
@@ -11776,10 +11823,10 @@
       <c r="Q19" s="30"/>
     </row>
     <row r="20" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I20" s="217"/>
-      <c r="J20" s="217"/>
-      <c r="K20" s="217"/>
-      <c r="L20" s="217"/>
+      <c r="I20" s="238"/>
+      <c r="J20" s="238"/>
+      <c r="K20" s="238"/>
+      <c r="L20" s="238"/>
       <c r="W20" s="29"/>
       <c r="X20" s="29"/>
     </row>
@@ -11954,15 +12001,15 @@
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B2" s="71"/>
-      <c r="C2" s="236" t="s">
+      <c r="C2" s="257" t="s">
         <v>252</v>
       </c>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
-      <c r="F2" s="236"/>
-      <c r="G2" s="236"/>
-      <c r="H2" s="236"/>
-      <c r="I2" s="236"/>
+      <c r="D2" s="257"/>
+      <c r="E2" s="257"/>
+      <c r="F2" s="257"/>
+      <c r="G2" s="257"/>
+      <c r="H2" s="257"/>
+      <c r="I2" s="257"/>
       <c r="J2" s="186"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
@@ -12003,7 +12050,7 @@
       <c r="G4" s="115"/>
       <c r="H4" s="115"/>
       <c r="I4" s="115"/>
-      <c r="J4" s="240" t="str">
+      <c r="J4" s="205" t="str">
         <f>IFERROR(AVERAGE(C4:I4),"Empty")</f>
         <v>Empty</v>
       </c>
@@ -12019,22 +12066,22 @@
       <c r="G5" s="115"/>
       <c r="H5" s="115"/>
       <c r="I5" s="115"/>
-      <c r="J5" s="240" t="str">
+      <c r="J5" s="205" t="str">
         <f>IFERROR(AVERAGE(C5:I5),"Empty")</f>
         <v>Empty</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="71"/>
-      <c r="C7" s="236" t="s">
+      <c r="C7" s="257" t="s">
         <v>253</v>
       </c>
-      <c r="D7" s="236"/>
-      <c r="E7" s="236"/>
-      <c r="F7" s="236"/>
-      <c r="G7" s="236"/>
-      <c r="H7" s="236"/>
-      <c r="I7" s="236"/>
+      <c r="D7" s="257"/>
+      <c r="E7" s="257"/>
+      <c r="F7" s="257"/>
+      <c r="G7" s="257"/>
+      <c r="H7" s="257"/>
+      <c r="I7" s="257"/>
       <c r="J7" s="88"/>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
@@ -12075,7 +12122,7 @@
       <c r="G9" s="115"/>
       <c r="H9" s="115"/>
       <c r="I9" s="115"/>
-      <c r="J9" s="240" t="str">
+      <c r="J9" s="205" t="str">
         <f>IFERROR(AVERAGE(C9:I9),"Empty")</f>
         <v>Empty</v>
       </c>
@@ -12091,7 +12138,7 @@
       <c r="G10" s="115"/>
       <c r="H10" s="115"/>
       <c r="I10" s="115"/>
-      <c r="J10" s="240" t="str">
+      <c r="J10" s="205" t="str">
         <f>IFERROR(AVERAGE(C10:I10),"Empty")</f>
         <v>Empty</v>
       </c>
@@ -12110,6 +12157,7 @@
   <dimension ref="B2:C32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="2.85546875" customWidth="1"/>
     <col min="2" max="2" width="21.85546875" customWidth="1"/>
     <col min="3" max="3" width="13.7109375" customWidth="1"/>
     <col min="4" max="4" width="1.7109375" customWidth="1"/>
@@ -12139,7 +12187,7 @@
       <c r="B5" s="96" t="s">
         <v>245</v>
       </c>
-      <c r="C5" s="240" t="str">
+      <c r="C5" s="205" t="str">
         <f>inf_flow_avg</f>
         <v>Empty</v>
       </c>
@@ -12148,7 +12196,7 @@
       <c r="B6" s="96" t="s">
         <v>246</v>
       </c>
-      <c r="C6" s="240">
+      <c r="C6" s="205">
         <f>inf_flow_max</f>
         <v>0</v>
       </c>
@@ -12157,7 +12205,7 @@
       <c r="B7" s="96" t="s">
         <v>247</v>
       </c>
-      <c r="C7" s="240">
+      <c r="C7" s="205">
         <f>basin_flow_total</f>
         <v>0</v>
       </c>
@@ -12166,7 +12214,7 @@
       <c r="B8" s="96" t="s">
         <v>248</v>
       </c>
-      <c r="C8" s="240">
+      <c r="C8" s="205">
         <f>clarifier_flow_total</f>
         <v>0</v>
       </c>
@@ -12175,7 +12223,7 @@
       <c r="B9" s="96" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="240">
+      <c r="C9" s="205">
         <f>clarifier_underflow_total</f>
         <v>0</v>
       </c>
@@ -12184,7 +12232,7 @@
       <c r="B10" s="96" t="s">
         <v>258</v>
       </c>
-      <c r="C10" s="240" t="str">
+      <c r="C10" s="205" t="str">
         <f>wasting_average</f>
         <v>Empty</v>
       </c>
@@ -12203,7 +12251,7 @@
       <c r="B13" s="73" t="s">
         <v>256</v>
       </c>
-      <c r="C13" s="238" t="str">
+      <c r="C13" s="203" t="str">
         <f>ph_daily_avg</f>
         <v>Empty</v>
       </c>
@@ -12221,7 +12269,7 @@
       <c r="B16" s="73" t="s">
         <v>109</v>
       </c>
-      <c r="C16" s="242">
+      <c r="C16" s="207">
         <f>Hourly!Q28</f>
         <v>0</v>
       </c>
@@ -12230,7 +12278,7 @@
       <c r="B17" s="28" t="s">
         <v>110</v>
       </c>
-      <c r="C17" s="243">
+      <c r="C17" s="208">
         <f>Hourly!Q30</f>
         <v>0</v>
       </c>
@@ -12245,28 +12293,28 @@
       <c r="C19" s="181"/>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B20" s="152" t="s">
+      <c r="B20" s="117" t="s">
         <v>242</v>
       </c>
-      <c r="C20" s="246" t="str">
+      <c r="C20" s="212" t="str">
         <f>lagoon_sludge_temp_avg</f>
         <v>Empty</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B21" s="161" t="s">
+      <c r="B21" s="117" t="s">
         <v>240</v>
       </c>
-      <c r="C21" s="250">
+      <c r="C21" s="212">
         <f>abf_tower_temperature</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B22" s="162" t="s">
+      <c r="B22" s="117" t="s">
         <v>241</v>
       </c>
-      <c r="C22" s="251">
+      <c r="C22" s="212">
         <f>aeration_basin_tempature</f>
         <v>0</v>
       </c>
@@ -12284,7 +12332,7 @@
       <c r="B25" s="177" t="s">
         <v>262</v>
       </c>
-      <c r="C25" s="248" t="str">
+      <c r="C25" s="212" t="str">
         <f>paa_daily_avg</f>
         <v>Empty</v>
       </c>
@@ -12293,7 +12341,7 @@
       <c r="B26" s="177" t="s">
         <v>263</v>
       </c>
-      <c r="C26" s="248" t="str">
+      <c r="C26" s="212" t="str">
         <f>paa_post_avg</f>
         <v>Empty</v>
       </c>
@@ -12311,7 +12359,7 @@
       <c r="B29" s="117" t="s">
         <v>243</v>
       </c>
-      <c r="C29" s="248" t="str">
+      <c r="C29" s="212" t="str">
         <f>aeration_basin_do_north_avg_handheld</f>
         <v>Empty</v>
       </c>
@@ -12320,7 +12368,7 @@
       <c r="B30" s="117" t="s">
         <v>244</v>
       </c>
-      <c r="C30" s="248" t="str">
+      <c r="C30" s="212" t="str">
         <f>aeration_basin_do_south_avg_handheld</f>
         <v>Empty</v>
       </c>
@@ -12329,7 +12377,7 @@
       <c r="B31" s="117" t="s">
         <v>260</v>
       </c>
-      <c r="C31" s="248" t="str">
+      <c r="C31" s="212" t="str">
         <f>aeration_basin_do_north_avg_probes</f>
         <v>Empty</v>
       </c>
@@ -12338,7 +12386,7 @@
       <c r="B32" s="117" t="s">
         <v>259</v>
       </c>
-      <c r="C32" s="248" t="str">
+      <c r="C32" s="212" t="str">
         <f>aeration_basin_do_south_avg_probes</f>
         <v>Empty</v>
       </c>
@@ -12845,11 +12893,52 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -12904,52 +12993,11 @@
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -13285,9 +13333,9 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FEF79AF6-431D-42B9-84BD-4FE9E9A3DF00}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D464854E-0460-4F1C-8C0F-FB6CF9126D7D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -13304,9 +13352,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D464854E-0460-4F1C-8C0F-FB6CF9126D7D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FEF79AF6-431D-42B9-84BD-4FE9E9A3DF00}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>